<commit_message>
Need to run F1=3 analysis
</commit_message>
<xml_diff>
--- a/BeatnotePostHotCellF1=4/Jul13,2026/Fit_ResultJun13.xlsx
+++ b/BeatnotePostHotCellF1=4/Jul13,2026/Fit_ResultJun13.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Diego\git\6s7p\BeatnotePostHotCellF1=4\Jul13,2026\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A4D51B92-9CB2-4667-BFB5-81795665ACFF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AF2E68B6-B6BA-43AC-9342-62BA58DBD7CC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{D9E101C5-8284-4B59-8B1C-2AD2D5F2FDD3}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="107" uniqueCount="40">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="106" uniqueCount="39">
   <si>
     <t>Date</t>
   </si>
@@ -156,9 +156,6 @@
   </si>
   <si>
     <t>Jul13,2026+5-39-08PM</t>
-  </si>
-  <si>
-    <t>Jul13,2026+12-46-48PM</t>
   </si>
 </sst>
 </file>
@@ -1387,7 +1384,7 @@
         <v>11</v>
       </c>
       <c r="B2" s="1">
-        <v>8.3363484131550397E-2</v>
+        <v>6.4896125092345797E-2</v>
       </c>
       <c r="C2" s="1">
         <v>1.6489052688978301</v>
@@ -1399,13 +1396,13 @@
         <v>-3.5883369219265799E-5</v>
       </c>
       <c r="F2" s="1">
-        <v>1.5655997494731799</v>
+        <v>1.50439839347147</v>
       </c>
       <c r="G2" s="1">
-        <v>39.888855590737997</v>
+        <v>39.841445316576802</v>
       </c>
       <c r="H2" s="1">
-        <v>1.04140829943926E-3</v>
+        <v>7.3249082742888195E-4</v>
       </c>
       <c r="L2" s="1"/>
     </row>
@@ -1414,7 +1411,7 @@
         <v>12</v>
       </c>
       <c r="B3" s="1">
-        <v>8.3757021233168596E-2</v>
+        <v>6.5241502827778394E-2</v>
       </c>
       <c r="C3" s="1">
         <v>1.6471156336470001</v>
@@ -1426,13 +1423,13 @@
         <v>-1.79977144130785E-4</v>
       </c>
       <c r="F3" s="1">
-        <v>2.0654154555297399</v>
+        <v>2.00419334592682</v>
       </c>
       <c r="G3" s="1">
-        <v>40.799759147066197</v>
+        <v>40.799754733238203</v>
       </c>
       <c r="H3" s="1">
-        <v>7.5221386507477695E-4</v>
+        <v>7.5221398477260803E-4</v>
       </c>
       <c r="L3" s="1"/>
     </row>
@@ -1441,7 +1438,7 @@
         <v>13</v>
       </c>
       <c r="B4" s="1">
-        <v>8.3417811249936594E-2</v>
+        <v>6.4980468998503793E-2</v>
       </c>
       <c r="C4" s="1">
         <v>1.64682653435071</v>
@@ -1453,13 +1450,13 @@
         <v>-1.56661092218066E-4</v>
       </c>
       <c r="F4" s="1">
-        <v>2.2747450298837002</v>
+        <v>2.2135504390041199</v>
       </c>
       <c r="G4" s="1">
-        <v>41.162763344932699</v>
+        <v>40.820715308662997</v>
       </c>
       <c r="H4" s="1">
-        <v>5.9320027741114397E-4</v>
+        <v>7.5221022377860601E-4</v>
       </c>
     </row>
     <row r="5" spans="1:20" ht="42.75">
@@ -1467,7 +1464,7 @@
         <v>14</v>
       </c>
       <c r="B5" s="1">
-        <v>8.4025870340482506E-2</v>
+        <v>6.5514217770456601E-2</v>
       </c>
       <c r="C5" s="1">
         <v>1.6472073470222099</v>
@@ -1479,13 +1476,13 @@
         <v>-3.8348484728154101E-4</v>
       </c>
       <c r="F5" s="1">
-        <v>1.8155824926617401</v>
+        <v>1.7543454543383099</v>
       </c>
       <c r="G5" s="1">
-        <v>40.829055315167203</v>
+        <v>41.183647345050701</v>
       </c>
       <c r="H5" s="1">
-        <v>7.5220872085382301E-4</v>
+        <v>1.15432129578544E-3</v>
       </c>
     </row>
     <row r="6" spans="1:20" ht="42.75">
@@ -1493,7 +1490,7 @@
         <v>15</v>
       </c>
       <c r="B6" s="1">
-        <v>8.2022959476588206E-2</v>
+        <v>6.3922916299629498E-2</v>
       </c>
       <c r="C6" s="1">
         <v>1.64695593343627</v>
@@ -1505,13 +1502,13 @@
         <v>-2.6589153950067601E-5</v>
       </c>
       <c r="F6" s="1">
-        <v>2.5240247955049702</v>
+        <v>2.4627785371180702</v>
       </c>
       <c r="G6" s="1">
-        <v>39.841850859595098</v>
+        <v>40.326145872444599</v>
       </c>
       <c r="H6" s="1">
-        <v>6.0913750818304105E-4</v>
+        <v>7.1636395727049998E-4</v>
       </c>
     </row>
     <row r="7" spans="1:20" ht="42.75">
@@ -1519,7 +1516,7 @@
         <v>16</v>
       </c>
       <c r="B7" s="1">
-        <v>8.3409466599106696E-2</v>
+        <v>6.4968524453632603E-2</v>
       </c>
       <c r="C7" s="1">
         <v>1.6501940896549401</v>
@@ -1531,13 +1528,13 @@
         <v>-1.8392707019857299E-4</v>
       </c>
       <c r="F7" s="1">
-        <v>1.5646194275512599</v>
+        <v>1.5034178939826801</v>
       </c>
       <c r="G7" s="1">
-        <v>40.356129216399601</v>
+        <v>40.3561048284921</v>
       </c>
       <c r="H7" s="1">
-        <v>7.5220657253493705E-4</v>
+        <v>7.5220490522947203E-4</v>
       </c>
     </row>
     <row r="8" spans="1:20" ht="42.75">
@@ -1545,7 +1542,7 @@
         <v>17</v>
       </c>
       <c r="B8" s="1">
-        <v>8.3177485471750606E-2</v>
+        <v>6.4822401873769905E-2</v>
       </c>
       <c r="C8" s="1">
         <v>1.650409194466</v>
@@ -1557,13 +1554,13 @@
         <v>1.47298933265976E-5</v>
       </c>
       <c r="F8" s="1">
-        <v>2.3159675365556298</v>
+        <v>2.2547214399647202</v>
       </c>
       <c r="G8" s="1">
-        <v>39.452890117896899</v>
+        <v>40.435776637143597</v>
       </c>
       <c r="H8" s="1">
-        <v>9.0763621270644899E-4</v>
+        <v>7.5221082557864203E-4</v>
       </c>
     </row>
     <row r="9" spans="1:20" ht="42.75">
@@ -1571,7 +1568,7 @@
         <v>18</v>
       </c>
       <c r="B9" s="1">
-        <v>8.3006037660706203E-2</v>
+        <v>6.4645386104361796E-2</v>
       </c>
       <c r="C9" s="1">
         <v>1.6511046344257601</v>
@@ -1583,13 +1580,13 @@
         <v>-4.6642466346437302E-5</v>
       </c>
       <c r="F9" s="1">
-        <v>2.3154761375400801</v>
+        <v>2.2542514178178998</v>
       </c>
       <c r="G9" s="1">
-        <v>40.4816455662842</v>
+        <v>39.891042790854499</v>
       </c>
       <c r="H9" s="1">
-        <v>7.5220995605928501E-4</v>
+        <v>8.9943553010377302E-4</v>
       </c>
     </row>
     <row r="10" spans="1:20" ht="42.75">
@@ -1597,7 +1594,7 @@
         <v>19</v>
       </c>
       <c r="B10" s="1">
-        <v>8.3019038948826299E-2</v>
+        <v>6.4722728337579E-2</v>
       </c>
       <c r="C10" s="1">
         <v>1.65173904312147</v>
@@ -1609,13 +1606,13 @@
         <v>-1.1828042711885701E-4</v>
       </c>
       <c r="F10" s="1">
-        <v>1.81485767952139</v>
+        <v>1.75363889067504</v>
       </c>
       <c r="G10" s="1">
-        <v>39.746959700973797</v>
+        <v>40.538851158397897</v>
       </c>
       <c r="H10" s="1">
-        <v>5.8624375927759204E-4</v>
+        <v>7.5221301947796205E-4</v>
       </c>
     </row>
     <row r="11" spans="1:20" ht="42.75">
@@ -1623,7 +1620,7 @@
         <v>20</v>
       </c>
       <c r="B11" s="1">
-        <v>8.3723462750931996E-2</v>
+        <v>6.5198191332667299E-2</v>
       </c>
       <c r="C11" s="1">
         <v>1.6491103552508199</v>
@@ -1635,13 +1632,13 @@
         <v>-2.30119837112956E-4</v>
       </c>
       <c r="F11" s="1">
-        <v>1.8145571051514899</v>
+        <v>1.7533619767689199</v>
       </c>
       <c r="G11" s="1">
-        <v>41.319569814947101</v>
+        <v>40.536141189137297</v>
       </c>
       <c r="H11" s="1">
-        <v>5.7862158210837103E-4</v>
+        <v>7.5220814089091805E-4</v>
       </c>
     </row>
     <row r="12" spans="1:20" ht="42.75">
@@ -1649,7 +1646,7 @@
         <v>21</v>
       </c>
       <c r="B12" s="1">
-        <v>8.3608574512507694E-2</v>
+        <v>6.5118995543562194E-2</v>
       </c>
       <c r="C12" s="1">
         <v>1.64866726512319</v>
@@ -1661,13 +1658,13 @@
         <v>-2.35305833877525E-4</v>
       </c>
       <c r="F12" s="1">
-        <v>2.31719396413739</v>
+        <v>2.2559915641938799</v>
       </c>
       <c r="G12" s="1">
-        <v>40.572826974018497</v>
+        <v>40.572882166146499</v>
       </c>
       <c r="H12" s="1">
-        <v>7.5220971883848797E-4</v>
+        <v>7.5222088547527096E-4</v>
       </c>
     </row>
     <row r="13" spans="1:20" ht="42.75">
@@ -1675,7 +1672,7 @@
         <v>22</v>
       </c>
       <c r="B13" s="1">
-        <v>8.3118939745191397E-2</v>
+        <v>6.4744655225756606E-2</v>
       </c>
       <c r="C13" s="1">
         <v>1.6484857954651999</v>
@@ -1687,13 +1684,13 @@
         <v>6.5475930703844804E-6</v>
       </c>
       <c r="F13" s="1">
-        <v>2.3125521492244898</v>
+        <v>2.2513330055590601</v>
       </c>
       <c r="G13" s="1">
-        <v>39.651822585186103</v>
+        <v>39.650528630462098</v>
       </c>
       <c r="H13" s="1">
-        <v>1.15564513145739E-3</v>
+        <v>1.1567964930471999E-3</v>
       </c>
     </row>
     <row r="14" spans="1:20" ht="42.75">
@@ -1701,7 +1698,7 @@
         <v>23</v>
       </c>
       <c r="B14" s="1">
-        <v>8.3605447355610901E-2</v>
+        <v>6.5055203385797997E-2</v>
       </c>
       <c r="C14" s="1">
         <v>1.6484666521959599</v>
@@ -1713,13 +1710,13 @@
         <v>-1.7639679029406901E-4</v>
       </c>
       <c r="F14" s="1">
-        <v>2.31506107539429</v>
+        <v>2.2538443117345901</v>
       </c>
       <c r="G14" s="1">
-        <v>41.468677251072201</v>
+        <v>40.674247999277497</v>
       </c>
       <c r="H14" s="1">
-        <v>1.0175731204911901E-3</v>
+        <v>7.52208993515213E-4</v>
       </c>
     </row>
     <row r="15" spans="1:20" ht="42.75">
@@ -1727,7 +1724,7 @@
         <v>24</v>
       </c>
       <c r="B15" s="1">
-        <v>8.3418150740260003E-2</v>
+        <v>6.4948449195513402E-2</v>
       </c>
       <c r="C15" s="1">
         <v>1.64897113077215</v>
@@ -1739,13 +1736,13 @@
         <v>-1.9285910341468101E-4</v>
       </c>
       <c r="F15" s="1">
-        <v>2.3156504037611301</v>
+        <v>2.2544456869006302</v>
       </c>
       <c r="G15" s="1">
-        <v>41.1326477554625</v>
+        <v>40.705348906219399</v>
       </c>
       <c r="H15" s="1">
-        <v>8.0797301489894495E-4</v>
+        <v>7.5221724454476401E-4</v>
       </c>
     </row>
     <row r="16" spans="1:20" ht="42.75">
@@ -1753,7 +1750,7 @@
         <v>25</v>
       </c>
       <c r="B16" s="1">
-        <v>8.3455841721042895E-2</v>
+        <v>6.4945497227791402E-2</v>
       </c>
       <c r="C16" s="1">
         <v>1.64937768743458</v>
@@ -1765,13 +1762,13 @@
         <v>-1.7462687930735999E-4</v>
       </c>
       <c r="F16" s="1">
-        <v>1.8153384255898399</v>
+        <v>1.7541266745699999</v>
       </c>
       <c r="G16" s="1">
-        <v>41.2921775392645</v>
+        <v>40.7181728306726</v>
       </c>
       <c r="H16" s="1">
-        <v>1.0498014455773599E-3</v>
+        <v>7.5220954969293797E-4</v>
       </c>
     </row>
     <row r="17" spans="1:8" ht="42.75">
@@ -1779,7 +1776,7 @@
         <v>26</v>
       </c>
       <c r="B17" s="1">
-        <v>8.3276939213918696E-2</v>
+        <v>6.4863395330163096E-2</v>
       </c>
       <c r="C17" s="1">
         <v>1.6489426317198701</v>
@@ -1791,352 +1788,336 @@
         <v>-1.6592203020265601E-4</v>
       </c>
       <c r="F17" s="1">
-        <v>2.3143359011743301</v>
+        <v>2.2531264155031399</v>
       </c>
       <c r="G17" s="1">
-        <v>40.718174794454697</v>
+        <v>39.764358533595797</v>
       </c>
       <c r="H17" s="1">
-        <v>7.5220824120456899E-4</v>
+        <v>1.1026591604233001E-3</v>
       </c>
     </row>
     <row r="18" spans="1:8" ht="42.75">
       <c r="A18" s="1" t="s">
-        <v>39</v>
+        <v>27</v>
       </c>
       <c r="B18" s="1">
-        <v>8.3521964118684094E-2</v>
+        <v>6.4713449109524701E-2</v>
       </c>
       <c r="C18" s="1">
-        <v>1.6499542479061</v>
-      </c>
-      <c r="D18" s="1">
-        <v>3.2339349386455201E-4</v>
+        <v>1.6481744217136001</v>
+      </c>
+      <c r="D18" s="2">
+        <v>6.7972185607939993E-5</v>
       </c>
       <c r="E18" s="1">
-        <v>-1.8555532057229501E-4</v>
+        <v>-1.2793985876687099E-4</v>
       </c>
       <c r="F18" s="1">
-        <v>1.5660432172549601</v>
+        <v>1.75326503269537</v>
       </c>
       <c r="G18" s="1">
-        <v>41.093662336661502</v>
+        <v>40.170611918737698</v>
       </c>
       <c r="H18" s="1">
-        <v>1.11661884809631E-3</v>
+        <v>7.6906148602765196E-4</v>
       </c>
     </row>
     <row r="19" spans="1:8" ht="42.75">
       <c r="A19" s="1" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B19" s="1">
-        <v>8.3116670967641595E-2</v>
+        <v>6.4825237757855897E-2</v>
       </c>
       <c r="C19" s="1">
-        <v>1.6481744217136001</v>
-      </c>
-      <c r="D19" s="2">
-        <v>6.7972185607939993E-5</v>
-      </c>
-      <c r="E19" s="1">
-        <v>-1.2793985876687099E-4</v>
+        <v>1.6465873748131099</v>
+      </c>
+      <c r="D19" s="1">
+        <v>2.57529520245287E-4</v>
+      </c>
+      <c r="E19" s="2">
+        <v>-7.0980137139593994E-5</v>
       </c>
       <c r="F19" s="1">
-        <v>1.8144543049298101</v>
+        <v>1.7551889206300999</v>
       </c>
       <c r="G19" s="1">
-        <v>40.766435572983802</v>
+        <v>40.845523906982599</v>
       </c>
       <c r="H19" s="1">
-        <v>7.5220962581331696E-4</v>
+        <v>7.5220777233973304E-4</v>
       </c>
     </row>
     <row r="20" spans="1:8" ht="42.75">
       <c r="A20" s="1" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="B20" s="1">
-        <v>8.3225256404970693E-2</v>
+        <v>6.4470305505123601E-2</v>
       </c>
       <c r="C20" s="1">
-        <v>1.6465873748131099</v>
+        <v>1.64618185252446</v>
       </c>
       <c r="D20" s="1">
-        <v>2.57529520245287E-4</v>
+        <v>1.9004085787397299E-4</v>
       </c>
       <c r="E20" s="2">
-        <v>-7.0980137139593994E-5</v>
+        <v>-2.2136627076530899E-5</v>
       </c>
       <c r="F20" s="1">
-        <v>1.8163848202022299</v>
+        <v>2.75426667909464</v>
       </c>
       <c r="G20" s="1">
-        <v>40.845529825129702</v>
+        <v>39.889892849373403</v>
       </c>
       <c r="H20" s="1">
-        <v>7.5220742643683296E-4</v>
+        <v>5.91059597309157E-4</v>
       </c>
     </row>
     <row r="21" spans="1:8" ht="42.75">
       <c r="A21" s="1" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B21" s="1">
-        <v>8.2797901589345094E-2</v>
+        <v>6.5433699222487096E-2</v>
       </c>
       <c r="C21" s="1">
-        <v>1.64618185252446</v>
+        <v>1.6468783109107299</v>
       </c>
       <c r="D21" s="1">
-        <v>1.9004085787397299E-4</v>
-      </c>
-      <c r="E21" s="2">
-        <v>-2.2136627076530899E-5</v>
+        <v>1.33300992379283E-3</v>
+      </c>
+      <c r="E21" s="1">
+        <v>-3.2264280559848201E-4</v>
       </c>
       <c r="F21" s="1">
-        <v>2.8154802128082301</v>
+        <v>2.2559095159999099</v>
       </c>
       <c r="G21" s="1">
-        <v>40.0355397136234</v>
+        <v>40.906917872165401</v>
       </c>
       <c r="H21" s="1">
-        <v>7.4803345106355299E-4</v>
+        <v>7.5220837551692396E-4</v>
       </c>
     </row>
     <row r="22" spans="1:8" ht="42.75">
       <c r="A22" s="1" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B22" s="1">
-        <v>8.4124029452458504E-2</v>
+        <v>6.4237906062167796E-2</v>
       </c>
       <c r="C22" s="1">
-        <v>1.6468783109107299</v>
+        <v>1.64777302981577</v>
       </c>
       <c r="D22" s="1">
-        <v>1.33300992379283E-3</v>
+        <v>6.8403317447661199E-4</v>
       </c>
       <c r="E22" s="1">
-        <v>-3.2264280559848201E-4</v>
+        <v>-1.61806308567992E-4</v>
       </c>
       <c r="F22" s="1">
-        <v>2.3171234125930198</v>
+        <v>2.5032163574863699</v>
       </c>
       <c r="G22" s="1">
-        <v>41.905853421350301</v>
+        <v>39.948779855544998</v>
       </c>
       <c r="H22" s="1">
-        <v>1.1563212932791599E-3</v>
+        <v>7.6388393414980799E-4</v>
       </c>
     </row>
     <row r="23" spans="1:8" ht="42.75">
       <c r="A23" s="1" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B23" s="1">
-        <v>8.2524964266572395E-2</v>
+        <v>6.51602437216873E-2</v>
       </c>
       <c r="C23" s="1">
-        <v>1.64777302981577</v>
+        <v>1.64661307141527</v>
       </c>
       <c r="D23" s="1">
-        <v>6.8403317447661199E-4</v>
+        <v>1.4544721931774899E-3</v>
       </c>
       <c r="E23" s="1">
-        <v>-1.61806308567992E-4</v>
+        <v>-2.6511739956727102E-4</v>
       </c>
       <c r="F23" s="1">
-        <v>2.5644332105527199</v>
+        <v>2.7137612957203201</v>
       </c>
       <c r="G23" s="1">
-        <v>40.920993329315003</v>
+        <v>40.935486681055004</v>
       </c>
       <c r="H23" s="1">
-        <v>7.5220830937307499E-4</v>
+        <v>6.9120867581541601E-4</v>
       </c>
     </row>
     <row r="24" spans="1:8" ht="42.75">
       <c r="A24" s="1" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="B24" s="1">
-        <v>8.3779837646985295E-2</v>
+        <v>6.4591400893665399E-2</v>
       </c>
       <c r="C24" s="1">
-        <v>1.64661307141527</v>
+        <v>1.64647748915448</v>
       </c>
       <c r="D24" s="1">
-        <v>1.4544721931774899E-3</v>
+        <v>7.5016398108375198E-4</v>
       </c>
       <c r="E24" s="1">
-        <v>-2.6511739956727102E-4</v>
+        <v>-1.4171338385419999E-4</v>
       </c>
       <c r="F24" s="1">
-        <v>2.7749714263410499</v>
+        <v>2.5022322732212601</v>
       </c>
       <c r="G24" s="1">
-        <v>41.922876774486099</v>
+        <v>40.440644286531402</v>
       </c>
       <c r="H24" s="1">
-        <v>1.1349406504848299E-3</v>
+        <v>9.9613005209969003E-4</v>
       </c>
     </row>
     <row r="25" spans="1:8" ht="42.75">
       <c r="A25" s="1" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="B25" s="1">
-        <v>8.2884597799815607E-2</v>
+        <v>6.4621020370609905E-2</v>
       </c>
       <c r="C25" s="1">
-        <v>1.64647748915448</v>
+        <v>1.6466076192117001</v>
       </c>
       <c r="D25" s="1">
-        <v>7.5016398108375198E-4</v>
+        <v>1.1285349524958999E-3</v>
       </c>
       <c r="E25" s="1">
-        <v>-1.4171338385419999E-4</v>
+        <v>-2.2444795525635599E-4</v>
       </c>
       <c r="F25" s="1">
-        <v>2.5634371622869399</v>
+        <v>2.0047659776812998</v>
       </c>
       <c r="G25" s="1">
-        <v>40.0104869607189</v>
+        <v>41.749517694573399</v>
       </c>
       <c r="H25" s="1">
-        <v>9.1169215716733001E-4</v>
+        <v>6.0499585182614802E-4</v>
       </c>
     </row>
     <row r="26" spans="1:8" ht="42.75">
       <c r="A26" s="1" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="B26" s="1">
-        <v>8.3056026546302203E-2</v>
+        <v>6.4713175919996493E-2</v>
       </c>
       <c r="C26" s="1">
-        <v>1.6466076192117001</v>
+        <v>1.6460373213117701</v>
       </c>
       <c r="D26" s="1">
-        <v>1.1285349524958999E-3</v>
+        <v>1.5195491112096201E-3</v>
       </c>
       <c r="E26" s="1">
-        <v>-2.2444795525635599E-4</v>
+        <v>-3.0803046884285998E-4</v>
       </c>
       <c r="F26" s="1">
-        <v>2.06596759228032</v>
+        <v>2.5053486406805199</v>
       </c>
       <c r="G26" s="1">
-        <v>41.9374478368306</v>
+        <v>40.066614858403803</v>
       </c>
       <c r="H26" s="1">
-        <v>1.1557044581734701E-3</v>
+        <v>8.2811674953733004E-4</v>
       </c>
     </row>
     <row r="27" spans="1:8" ht="42.75">
       <c r="A27" s="1" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B27" s="1">
-        <v>8.3119909910801301E-2</v>
+        <v>6.4608197537483703E-2</v>
       </c>
       <c r="C27" s="1">
-        <v>1.6460373213117701</v>
+        <v>1.64463491274189</v>
       </c>
       <c r="D27" s="1">
-        <v>1.5195491112096201E-3</v>
+        <v>6.2658825883887598E-4</v>
       </c>
       <c r="E27" s="1">
-        <v>-3.0803046884285998E-4</v>
+        <v>-1.5362762784175399E-4</v>
       </c>
       <c r="F27" s="1">
-        <v>2.5665670108013701</v>
+        <v>1.8347590513925001</v>
       </c>
       <c r="G27" s="1">
-        <v>40.951611098991499</v>
+        <v>41.839977199731401</v>
       </c>
       <c r="H27" s="1">
-        <v>7.5220819426450496E-4</v>
+        <v>6.0029900465471205E-4</v>
       </c>
     </row>
     <row r="28" spans="1:8" ht="42.75">
       <c r="A28" s="1" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B28" s="1">
-        <v>8.29152163470048E-2</v>
+        <v>6.4507451500493501E-2</v>
       </c>
       <c r="C28" s="1">
-        <v>1.64463491274189</v>
+        <v>1.6445019588141601</v>
       </c>
       <c r="D28" s="1">
-        <v>6.2658825883887598E-4</v>
+        <v>8.2620117838240199E-4</v>
       </c>
       <c r="E28" s="1">
-        <v>-1.5362762784175399E-4</v>
+        <v>-1.31340818125899E-4</v>
       </c>
       <c r="F28" s="1">
-        <v>1.8959371752588301</v>
+        <v>2.58392102339036</v>
       </c>
       <c r="G28" s="1">
-        <v>40.999521283361503</v>
+        <v>41.0152864056002</v>
       </c>
       <c r="H28" s="1">
-        <v>7.5220813112782299E-4</v>
+        <v>7.5220771155717903E-4</v>
       </c>
     </row>
     <row r="29" spans="1:8" ht="42.75">
       <c r="A29" s="1" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="B29" s="1">
-        <v>8.28084692004942E-2</v>
+        <v>6.4884214968972106E-2</v>
       </c>
       <c r="C29" s="1">
-        <v>1.6445019588141601</v>
+        <v>1.64580515169229</v>
       </c>
       <c r="D29" s="1">
-        <v>8.2620117838240199E-4</v>
+        <v>1.4896118497053799E-3</v>
       </c>
       <c r="E29" s="1">
-        <v>-1.31340818125899E-4</v>
+        <v>-3.3275212705288098E-4</v>
       </c>
       <c r="F29" s="1">
-        <v>2.6451261477933099</v>
+        <v>1.83525278377538</v>
       </c>
       <c r="G29" s="1">
-        <v>41.015308316162098</v>
+        <v>41.005453916708703</v>
       </c>
       <c r="H29" s="1">
-        <v>7.5220928079247499E-4</v>
-      </c>
-    </row>
-    <row r="30" spans="1:8" ht="42.75">
-      <c r="A30" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="B30" s="1">
-        <v>8.3334028420614895E-2</v>
-      </c>
-      <c r="C30" s="1">
-        <v>1.64580515169229</v>
-      </c>
-      <c r="D30" s="1">
-        <v>1.4896118497053799E-3</v>
-      </c>
-      <c r="E30" s="1">
-        <v>-3.3275212705288098E-4</v>
-      </c>
-      <c r="F30" s="1">
-        <v>1.8964690380839999</v>
-      </c>
-      <c r="G30" s="1">
-        <v>42.0019358175104</v>
-      </c>
-      <c r="H30" s="1">
-        <v>5.7878667261706802E-4</v>
-      </c>
+        <v>7.5220844896903998E-4</v>
+      </c>
+    </row>
+    <row r="30" spans="1:8">
+      <c r="A30" s="1"/>
+      <c r="B30" s="1"/>
+      <c r="C30" s="1"/>
+      <c r="D30" s="1"/>
+      <c r="E30" s="1"/>
+      <c r="F30" s="1"/>
+      <c r="G30" s="1"/>
+      <c r="H30" s="1"/>
     </row>
     <row r="31" spans="1:8">
       <c r="A31" s="1"/>
@@ -2218,7 +2199,7 @@
   <dimension ref="A1:P37"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
-    <row r="1" spans="1:8">
+    <row r="1" spans="1:11">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2228,8 +2209,10 @@
       <c r="C1" s="1" t="s">
         <v>4</v>
       </c>
-    </row>
-    <row r="2" spans="1:8" ht="42.75">
+      <c r="J1" s="1"/>
+      <c r="K1" s="1"/>
+    </row>
+    <row r="2" spans="1:11" ht="42.75">
       <c r="A2" s="1" t="s">
         <v>16</v>
       </c>
@@ -2237,10 +2220,11 @@
         <v>4.0279639492061596</v>
       </c>
       <c r="C2" s="1">
-        <v>8.3409466599106696E-2</v>
-      </c>
-    </row>
-    <row r="3" spans="1:8" ht="42.75">
+        <v>6.4968524453632603E-2</v>
+      </c>
+      <c r="J2" s="1"/>
+    </row>
+    <row r="3" spans="1:11" ht="42.75">
       <c r="A3" s="1" t="s">
         <v>17</v>
       </c>
@@ -2248,7 +2232,7 @@
         <v>4.0667523488381301</v>
       </c>
       <c r="C3" s="1">
-        <v>8.3177485471750606E-2</v>
+        <v>6.4822401873769905E-2</v>
       </c>
       <c r="G3">
         <v>894</v>
@@ -2256,8 +2240,9 @@
       <c r="H3">
         <v>456</v>
       </c>
-    </row>
-    <row r="4" spans="1:8" ht="42.75">
+      <c r="J3" s="1"/>
+    </row>
+    <row r="4" spans="1:11" ht="42.75">
       <c r="A4" s="1" t="s">
         <v>18</v>
       </c>
@@ -2265,7 +2250,7 @@
         <v>4.0183878243548996</v>
       </c>
       <c r="C4" s="1">
-        <v>8.3006037660706203E-2</v>
+        <v>6.4645386104361796E-2</v>
       </c>
       <c r="F4" t="s">
         <v>1</v>
@@ -2276,10 +2261,11 @@
       </c>
       <c r="H4">
         <f>AVERAGE(C2:C29)</f>
-        <v>8.3253337132306662E-2</v>
-      </c>
-    </row>
-    <row r="5" spans="1:8" ht="42.75">
+        <v>6.483410577033491E-2</v>
+      </c>
+      <c r="J4" s="1"/>
+    </row>
+    <row r="5" spans="1:11" ht="42.75">
       <c r="A5" s="1" t="s">
         <v>19</v>
       </c>
@@ -2287,7 +2273,7 @@
         <v>4.0314213938624102</v>
       </c>
       <c r="C5" s="1">
-        <v>8.3019038948826299E-2</v>
+        <v>6.4722728337579E-2</v>
       </c>
       <c r="F5" t="s">
         <v>2</v>
@@ -2298,10 +2284,11 @@
       </c>
       <c r="H5">
         <f>_xlfn.STDEV.S(C2:C29)</f>
-        <v>4.4770424937099043E-4</v>
-      </c>
-    </row>
-    <row r="6" spans="1:8" ht="42.75">
+        <v>3.3855545798518768E-4</v>
+      </c>
+      <c r="J5" s="1"/>
+    </row>
+    <row r="6" spans="1:11" ht="42.75">
       <c r="A6" s="1" t="s">
         <v>20</v>
       </c>
@@ -2309,7 +2296,7 @@
         <v>4.0505545969773804</v>
       </c>
       <c r="C6" s="1">
-        <v>8.3723462750931996E-2</v>
+        <v>6.5198191332667299E-2</v>
       </c>
       <c r="F6" t="s">
         <v>3</v>
@@ -2320,10 +2307,11 @@
       </c>
       <c r="H6">
         <f>H5/H4/SQRT(COUNT(C2:C29))</f>
-        <v>1.0162733801804158E-3</v>
-      </c>
-    </row>
-    <row r="7" spans="1:8" ht="42.75">
+        <v>9.8684121375140874E-4</v>
+      </c>
+      <c r="J6" s="1"/>
+    </row>
+    <row r="7" spans="1:11" ht="42.75">
       <c r="A7" s="1" t="s">
         <v>21</v>
       </c>
@@ -2331,10 +2319,11 @@
         <v>4.0517862191438496</v>
       </c>
       <c r="C7" s="1">
-        <v>8.3608574512507694E-2</v>
-      </c>
-    </row>
-    <row r="8" spans="1:8" ht="42.75">
+        <v>6.5118995543562194E-2</v>
+      </c>
+      <c r="J7" s="1"/>
+    </row>
+    <row r="8" spans="1:11" ht="42.75">
       <c r="A8" s="1" t="s">
         <v>22</v>
       </c>
@@ -2342,10 +2331,11 @@
         <v>4.0424645012040497</v>
       </c>
       <c r="C8" s="1">
-        <v>8.3118939745191397E-2</v>
-      </c>
-    </row>
-    <row r="9" spans="1:8" ht="42.75">
+        <v>6.4744655225756606E-2</v>
+      </c>
+      <c r="J8" s="1"/>
+    </row>
+    <row r="9" spans="1:11" ht="42.75">
       <c r="A9" s="1" t="s">
         <v>23</v>
       </c>
@@ -2353,10 +2343,11 @@
         <v>4.0243487276243002</v>
       </c>
       <c r="C9" s="1">
-        <v>8.3605447355610901E-2</v>
-      </c>
-    </row>
-    <row r="10" spans="1:8" ht="42.75">
+        <v>6.5055203385797997E-2</v>
+      </c>
+      <c r="J9" s="1"/>
+    </row>
+    <row r="10" spans="1:11" ht="42.75">
       <c r="A10" s="1" t="s">
         <v>24</v>
       </c>
@@ -2364,10 +2355,11 @@
         <v>4.0367409025359304</v>
       </c>
       <c r="C10" s="1">
-        <v>8.3418150740260003E-2</v>
-      </c>
-    </row>
-    <row r="11" spans="1:8" ht="42.75">
+        <v>6.4948449195513402E-2</v>
+      </c>
+      <c r="J10" s="1"/>
+    </row>
+    <row r="11" spans="1:11" ht="42.75">
       <c r="A11" s="1" t="s">
         <v>25</v>
       </c>
@@ -2375,10 +2367,11 @@
         <v>4.0491156124478902</v>
       </c>
       <c r="C11" s="1">
-        <v>8.3455841721042895E-2</v>
-      </c>
-    </row>
-    <row r="12" spans="1:8" ht="42.75">
+        <v>6.4945497227791402E-2</v>
+      </c>
+      <c r="J11" s="1"/>
+    </row>
+    <row r="12" spans="1:11" ht="42.75">
       <c r="A12" s="1" t="s">
         <v>26</v>
       </c>
@@ -2386,10 +2379,11 @@
         <v>4.0406778045491096</v>
       </c>
       <c r="C12" s="1">
-        <v>8.3276939213918696E-2</v>
-      </c>
-    </row>
-    <row r="13" spans="1:8" ht="42.75">
+        <v>6.4863395330163096E-2</v>
+      </c>
+      <c r="J12" s="1"/>
+    </row>
+    <row r="13" spans="1:11" ht="42.75">
       <c r="A13" s="1" t="s">
         <v>27</v>
       </c>
@@ -2397,10 +2391,11 @@
         <v>4.0437611760653196</v>
       </c>
       <c r="C13" s="1">
-        <v>8.3116670967641595E-2</v>
-      </c>
-    </row>
-    <row r="14" spans="1:8" ht="42.75">
+        <v>6.4713449109524701E-2</v>
+      </c>
+      <c r="J13" s="1"/>
+    </row>
+    <row r="14" spans="1:11" ht="42.75">
       <c r="A14" s="1" t="s">
         <v>11</v>
       </c>
@@ -2408,10 +2403,11 @@
         <v>4.0356877834891698</v>
       </c>
       <c r="C14" s="1">
-        <v>8.3363484131550397E-2</v>
-      </c>
-    </row>
-    <row r="15" spans="1:8" ht="42.75">
+        <v>6.4896125092345797E-2</v>
+      </c>
+      <c r="J14" s="1"/>
+    </row>
+    <row r="15" spans="1:11" ht="42.75">
       <c r="A15" s="1" t="s">
         <v>12</v>
       </c>
@@ -2419,10 +2415,11 @@
         <v>4.0543291932026699</v>
       </c>
       <c r="C15" s="1">
-        <v>8.3757021233168596E-2</v>
-      </c>
-    </row>
-    <row r="16" spans="1:8" ht="42.75">
+        <v>6.5241502827778394E-2</v>
+      </c>
+      <c r="J15" s="1"/>
+    </row>
+    <row r="16" spans="1:11" ht="42.75">
       <c r="A16" s="1" t="s">
         <v>13</v>
       </c>
@@ -2430,8 +2427,9 @@
         <v>4.0440448461837999</v>
       </c>
       <c r="C16" s="1">
-        <v>8.3417811249936594E-2</v>
-      </c>
+        <v>6.4980468998503793E-2</v>
+      </c>
+      <c r="J16" s="1"/>
     </row>
     <row r="17" spans="1:16" ht="42.75">
       <c r="A17" s="1" t="s">
@@ -2441,8 +2439,9 @@
         <v>4.0482658159189198</v>
       </c>
       <c r="C17" s="1">
-        <v>8.4025870340482506E-2</v>
-      </c>
+        <v>6.5514217770456601E-2</v>
+      </c>
+      <c r="J17" s="1"/>
     </row>
     <row r="18" spans="1:16" ht="42.75">
       <c r="A18" s="1" t="s">
@@ -2452,8 +2451,9 @@
         <v>4.0372658698111801</v>
       </c>
       <c r="C18" s="1">
-        <v>8.2022959476588206E-2</v>
-      </c>
+        <v>6.3922916299629498E-2</v>
+      </c>
+      <c r="J18" s="1"/>
     </row>
     <row r="19" spans="1:16" ht="42.75">
       <c r="A19" s="1" t="s">
@@ -2463,8 +2463,9 @@
         <v>4.0430873829414802</v>
       </c>
       <c r="C19" s="1">
-        <v>8.3225256404970693E-2</v>
-      </c>
+        <v>6.4825237757855897E-2</v>
+      </c>
+      <c r="J19" s="1"/>
     </row>
     <row r="20" spans="1:16" ht="42.75">
       <c r="A20" s="1" t="s">
@@ -2474,8 +2475,9 @@
         <v>4.0311378792119203</v>
       </c>
       <c r="C20" s="1">
-        <v>8.2797901589345094E-2</v>
-      </c>
+        <v>6.4470305505123601E-2</v>
+      </c>
+      <c r="J20" s="1"/>
     </row>
     <row r="21" spans="1:16" ht="42.75">
       <c r="A21" s="1" t="s">
@@ -2485,8 +2487,9 @@
         <v>4.01331392262989</v>
       </c>
       <c r="C21" s="1">
-        <v>8.4124029452458504E-2</v>
-      </c>
+        <v>6.5433699222487096E-2</v>
+      </c>
+      <c r="J21" s="1"/>
     </row>
     <row r="22" spans="1:16" ht="42.75">
       <c r="A22" s="1" t="s">
@@ -2496,8 +2499,9 @@
         <v>4.0578910745577002</v>
       </c>
       <c r="C22" s="1">
-        <v>8.2524964266572395E-2</v>
-      </c>
+        <v>6.4237906062167796E-2</v>
+      </c>
+      <c r="J22" s="1"/>
     </row>
     <row r="23" spans="1:16" ht="42.75">
       <c r="A23" s="1" t="s">
@@ -2507,8 +2511,9 @@
         <v>4.02794326730218</v>
       </c>
       <c r="C23" s="1">
-        <v>8.3779837646985295E-2</v>
-      </c>
+        <v>6.51602437216873E-2</v>
+      </c>
+      <c r="J23" s="1"/>
     </row>
     <row r="24" spans="1:16" ht="42.75">
       <c r="A24" s="1" t="s">
@@ -2518,8 +2523,9 @@
         <v>4.0616651770599299</v>
       </c>
       <c r="C24" s="1">
-        <v>8.2884597799815607E-2</v>
-      </c>
+        <v>6.4591400893665399E-2</v>
+      </c>
+      <c r="J24" s="1"/>
     </row>
     <row r="25" spans="1:16" ht="42.75">
       <c r="A25" s="1" t="s">
@@ -2529,8 +2535,9 @@
         <v>4.02065487780051</v>
       </c>
       <c r="C25" s="1">
-        <v>8.3056026546302203E-2</v>
-      </c>
+        <v>6.4621020370609905E-2</v>
+      </c>
+      <c r="J25" s="1"/>
     </row>
     <row r="26" spans="1:16" ht="42.75">
       <c r="A26" s="1" t="s">
@@ -2540,8 +2547,9 @@
         <v>4.0194143809069702</v>
       </c>
       <c r="C26" s="1">
-        <v>8.3119909910801301E-2</v>
-      </c>
+        <v>6.4713175919996493E-2</v>
+      </c>
+      <c r="J26" s="1"/>
     </row>
     <row r="27" spans="1:16" ht="42.75">
       <c r="A27" s="1" t="s">
@@ -2551,8 +2559,9 @@
         <v>4.0195181922825496</v>
       </c>
       <c r="C27" s="1">
-        <v>8.29152163470048E-2</v>
-      </c>
+        <v>6.4608197537483703E-2</v>
+      </c>
+      <c r="J27" s="1"/>
     </row>
     <row r="28" spans="1:16" ht="42.75">
       <c r="A28" s="1" t="s">
@@ -2562,8 +2571,9 @@
         <v>4.0060394450385299</v>
       </c>
       <c r="C28" s="1">
-        <v>8.28084692004942E-2</v>
-      </c>
+        <v>6.4507451500493501E-2</v>
+      </c>
+      <c r="J28" s="1"/>
     </row>
     <row r="29" spans="1:16" ht="42.75">
       <c r="A29" s="1" t="s">
@@ -2573,13 +2583,16 @@
         <v>4.03113906858741</v>
       </c>
       <c r="C29" s="1">
-        <v>8.3334028420614895E-2</v>
-      </c>
+        <v>6.4884214968972106E-2</v>
+      </c>
+      <c r="J29" s="1"/>
     </row>
     <row r="30" spans="1:16">
       <c r="A30" s="1"/>
       <c r="B30" s="1"/>
       <c r="C30" s="1"/>
+      <c r="J30" s="1"/>
+      <c r="K30" s="1"/>
       <c r="N30" s="1"/>
       <c r="O30" s="1"/>
       <c r="P30" s="1"/>
@@ -2588,6 +2601,8 @@
       <c r="A31" s="1"/>
       <c r="B31" s="1"/>
       <c r="C31" s="1"/>
+      <c r="J31" s="1"/>
+      <c r="K31" s="1"/>
       <c r="N31" s="1"/>
       <c r="O31" s="1"/>
       <c r="P31" s="1"/>
@@ -2596,6 +2611,8 @@
       <c r="A32" s="1"/>
       <c r="B32" s="1"/>
       <c r="C32" s="1"/>
+      <c r="J32" s="1"/>
+      <c r="K32" s="1"/>
       <c r="N32" s="1"/>
       <c r="O32" s="1"/>
       <c r="P32" s="1"/>
@@ -2604,6 +2621,8 @@
       <c r="A33" s="1"/>
       <c r="B33" s="1"/>
       <c r="C33" s="1"/>
+      <c r="J33" s="1"/>
+      <c r="K33" s="1"/>
       <c r="N33" s="1"/>
       <c r="O33" s="1"/>
       <c r="P33" s="1"/>
@@ -2612,6 +2631,8 @@
       <c r="A34" s="1"/>
       <c r="B34" s="1"/>
       <c r="C34" s="1"/>
+      <c r="J34" s="1"/>
+      <c r="K34" s="1"/>
       <c r="N34" s="1"/>
       <c r="O34" s="1"/>
       <c r="P34" s="1"/>
@@ -2620,6 +2641,8 @@
       <c r="A35" s="1"/>
       <c r="B35" s="1"/>
       <c r="C35" s="1"/>
+      <c r="J35" s="1"/>
+      <c r="K35" s="1"/>
       <c r="N35" s="1"/>
       <c r="O35" s="1"/>
       <c r="P35" s="1"/>
@@ -2628,12 +2651,16 @@
       <c r="A36" s="1"/>
       <c r="B36" s="1"/>
       <c r="C36" s="1"/>
+      <c r="J36" s="1"/>
+      <c r="K36" s="1"/>
       <c r="N36" s="1"/>
       <c r="O36" s="1"/>
       <c r="P36" s="1"/>
     </row>
     <row r="37" spans="1:16">
       <c r="C37" s="1"/>
+      <c r="J37" s="1"/>
+      <c r="K37" s="1"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>